<commit_message>
1차 실험 완료 (SR, GCR)
</commit_message>
<xml_diff>
--- a/FP403_result.xlsx
+++ b/FP403_result.xlsx
@@ -482,21 +482,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Put Toiletpaper in the cabinet</t>
+          <t>Put Plunger in the cabinet and Put the PaperTowelRoll on the countertop</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>FAILED (Execution Errors)</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>